<commit_message>
Yaro | improving readability
</commit_message>
<xml_diff>
--- a/Dataset/N2OR.xlsx
+++ b/Dataset/N2OR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10302"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pylya\Desktop\PhD\PhD\CSP_Solver_Final\Dataset\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/uk45965245/Documents/CoSPLib/Dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{233E796B-9693-4772-9D6A-7086BA055E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7428037-F860-EE46-AABF-82EFA592CE9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30240" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="790" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="parameters" sheetId="1" r:id="rId1"/>
@@ -251,20 +251,6 @@
     <t>Optimisation</t>
   </si>
   <si>
-    <r>
-      <t>NEW19A3731</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Roboto Light"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
     <t>NEW19A3739</t>
   </si>
   <si>
@@ -440,13 +426,16 @@
   </si>
   <si>
     <t>P34</t>
+  </si>
+  <si>
+    <t>NEW19A3731</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -485,12 +474,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Roboto Light"/>
     </font>
     <font>
       <sz val="10"/>
@@ -617,16 +600,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -931,13 +914,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="35.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="27.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -948,12 +931,12 @@
       </c>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>3</v>
@@ -962,7 +945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
@@ -974,7 +957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -988,7 +971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
@@ -996,13 +979,13 @@
         <v>0.89583333333333337</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E5" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>17</v>
       </c>
@@ -1014,7 +997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
@@ -1028,7 +1011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>8</v>
       </c>
@@ -1042,7 +1025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>18</v>
       </c>
@@ -1056,7 +1039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>19</v>
       </c>
@@ -1068,7 +1051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
@@ -1082,7 +1065,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D12" s="4" t="s">
         <v>14</v>
       </c>
@@ -1090,7 +1073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D13" s="4" t="s">
         <v>21</v>
       </c>
@@ -1098,7 +1081,7 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D14" s="4" t="s">
         <v>15</v>
       </c>
@@ -1106,7 +1089,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D15" s="4" t="s">
         <v>22</v>
       </c>
@@ -1114,7 +1097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="D16" s="4" t="s">
         <v>23</v>
       </c>
@@ -1122,7 +1105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="4:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:5" x14ac:dyDescent="0.2">
       <c r="D17" s="4" t="s">
         <v>16</v>
       </c>
@@ -1138,20 +1121,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65C69255-5912-4D6E-83E6-D37C87DA9D15}">
   <dimension ref="A1:P157"/>
-  <sheetFormatPr defaultColWidth="9.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.33203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" style="15" customWidth="1"/>
+    <col min="1" max="1" width="14.5" style="15" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" style="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.33203125" style="16" customWidth="1"/>
     <col min="4" max="5" width="9.33203125" style="16"/>
-    <col min="6" max="6" width="16.44140625" style="15" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.5" style="15" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" style="15" customWidth="1"/>
     <col min="8" max="11" width="9.33203125" style="16"/>
-    <col min="12" max="12" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="9.33203125" style="17"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="14" customFormat="1" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" s="14" customFormat="1" ht="29.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
         <v>24</v>
       </c>
@@ -1168,7 +1151,7 @@
         <v>28</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G1" s="11" t="s">
         <v>29</v>
@@ -1198,7 +1181,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="15" t="s">
         <v>38</v>
       </c>
@@ -1212,10 +1195,10 @@
         <v>0</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G2" s="17"/>
       <c r="L2" s="16"/>
@@ -1224,7 +1207,7 @@
       <c r="O2" s="16"/>
       <c r="P2" s="16"/>
     </row>
-    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="15" t="s">
         <v>40</v>
       </c>
@@ -1238,10 +1221,10 @@
         <v>0</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G3" s="17"/>
       <c r="L3" s="16"/>
@@ -1250,7 +1233,7 @@
       <c r="O3" s="16"/>
       <c r="P3" s="16"/>
     </row>
-    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="15" t="s">
         <v>41</v>
       </c>
@@ -1264,10 +1247,10 @@
         <v>0</v>
       </c>
       <c r="E4" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G4" s="17"/>
       <c r="L4" s="16"/>
@@ -1276,7 +1259,7 @@
       <c r="O4" s="16"/>
       <c r="P4" s="16"/>
     </row>
-    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="15" t="s">
         <v>42</v>
       </c>
@@ -1290,10 +1273,10 @@
         <v>0</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G5" s="17"/>
       <c r="L5" s="16"/>
@@ -1302,7 +1285,7 @@
       <c r="O5" s="16"/>
       <c r="P5" s="16"/>
     </row>
-    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="15" t="s">
         <v>43</v>
       </c>
@@ -1316,10 +1299,10 @@
         <v>0</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G6" s="17"/>
       <c r="L6" s="16"/>
@@ -1328,7 +1311,7 @@
       <c r="O6" s="16"/>
       <c r="P6" s="16"/>
     </row>
-    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="15" t="s">
         <v>44</v>
       </c>
@@ -1342,10 +1325,10 @@
         <v>0</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G7" s="17"/>
       <c r="L7" s="16"/>
@@ -1354,7 +1337,7 @@
       <c r="O7" s="16"/>
       <c r="P7" s="16"/>
     </row>
-    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="15" t="s">
         <v>46</v>
       </c>
@@ -1368,10 +1351,10 @@
         <v>0</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G8" s="17"/>
       <c r="J8" s="16">
@@ -1386,7 +1369,7 @@
       <c r="O8" s="16"/>
       <c r="P8" s="16"/>
     </row>
-    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="15" t="s">
         <v>47</v>
       </c>
@@ -1400,10 +1383,10 @@
         <v>0</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G9" s="17"/>
       <c r="L9" s="16"/>
@@ -1412,7 +1395,7 @@
       <c r="O9" s="16"/>
       <c r="P9" s="16"/>
     </row>
-    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="15" t="s">
         <v>48</v>
       </c>
@@ -1426,13 +1409,13 @@
         <v>0</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F10" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="G10" s="17" t="s">
         <v>99</v>
-      </c>
-      <c r="G10" s="17" t="s">
-        <v>100</v>
       </c>
       <c r="L10" s="16"/>
       <c r="M10" s="16"/>
@@ -1440,7 +1423,7 @@
       <c r="O10" s="16"/>
       <c r="P10" s="16"/>
     </row>
-    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="15" t="s">
         <v>49</v>
       </c>
@@ -1454,10 +1437,10 @@
         <v>0</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G11" s="17"/>
       <c r="L11" s="16"/>
@@ -1466,7 +1449,7 @@
       <c r="O11" s="16"/>
       <c r="P11" s="16"/>
     </row>
-    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="15" t="s">
         <v>50</v>
       </c>
@@ -1480,10 +1463,10 @@
         <v>0</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G12" s="17"/>
       <c r="H12" s="16">
@@ -1498,7 +1481,7 @@
       <c r="O12" s="16"/>
       <c r="P12" s="16"/>
     </row>
-    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="15" t="s">
         <v>52</v>
       </c>
@@ -1512,10 +1495,10 @@
         <v>0</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G13" s="17"/>
       <c r="H13" s="16">
@@ -1530,7 +1513,7 @@
       <c r="O13" s="16"/>
       <c r="P13" s="16"/>
     </row>
-    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="15" t="s">
         <v>53</v>
       </c>
@@ -1544,10 +1527,10 @@
         <v>0</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G14" s="17"/>
       <c r="L14" s="16"/>
@@ -1556,7 +1539,7 @@
       <c r="O14" s="16"/>
       <c r="P14" s="16"/>
     </row>
-    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="15" t="s">
         <v>54</v>
       </c>
@@ -1570,10 +1553,10 @@
         <v>0</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G15" s="17"/>
       <c r="L15" s="16"/>
@@ -1582,7 +1565,7 @@
       <c r="O15" s="16"/>
       <c r="P15" s="16"/>
     </row>
-    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="15" t="s">
         <v>56</v>
       </c>
@@ -1596,13 +1579,13 @@
         <v>0</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F16" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="G16" s="17" t="s">
         <v>106</v>
-      </c>
-      <c r="G16" s="17" t="s">
-        <v>107</v>
       </c>
       <c r="L16" s="16"/>
       <c r="M16" s="16"/>
@@ -1610,7 +1593,7 @@
       <c r="O16" s="16"/>
       <c r="P16" s="16"/>
     </row>
-    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="15" t="s">
         <v>57</v>
       </c>
@@ -1624,10 +1607,10 @@
         <v>0</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G17" s="17"/>
       <c r="L17" s="16"/>
@@ -1636,7 +1619,7 @@
       <c r="O17" s="16"/>
       <c r="P17" s="16"/>
     </row>
-    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="15" t="s">
         <v>58</v>
       </c>
@@ -1650,10 +1633,10 @@
         <v>0</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G18" s="17"/>
       <c r="L18" s="16"/>
@@ -1662,7 +1645,7 @@
       <c r="O18" s="16"/>
       <c r="P18" s="16"/>
     </row>
-    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="15" t="s">
         <v>59</v>
       </c>
@@ -1676,10 +1659,10 @@
         <v>1</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J19" s="16">
         <v>1</v>
@@ -1692,7 +1675,7 @@
       <c r="N19" s="16"/>
       <c r="O19" s="16"/>
     </row>
-    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="15" t="s">
         <v>61</v>
       </c>
@@ -1706,17 +1689,17 @@
         <v>0</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="L20" s="16"/>
       <c r="M20" s="16"/>
       <c r="N20" s="16"/>
       <c r="O20" s="16"/>
     </row>
-    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="15" t="s">
         <v>62</v>
       </c>
@@ -1730,20 +1713,20 @@
         <v>0</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F21" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="G21" s="15" t="s">
         <v>112</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>113</v>
       </c>
       <c r="L21" s="16"/>
       <c r="M21" s="16"/>
       <c r="N21" s="16"/>
       <c r="O21" s="16"/>
     </row>
-    <row r="22" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="15" t="s">
         <v>63</v>
       </c>
@@ -1757,20 +1740,20 @@
         <v>0</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F22" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="G22" s="15" t="s">
         <v>114</v>
-      </c>
-      <c r="G22" s="15" t="s">
-        <v>115</v>
       </c>
       <c r="L22" s="16"/>
       <c r="M22" s="16"/>
       <c r="N22" s="16"/>
       <c r="O22" s="16"/>
     </row>
-    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="15" t="s">
         <v>64</v>
       </c>
@@ -1784,17 +1767,17 @@
         <v>0</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L23" s="16"/>
       <c r="M23" s="16"/>
       <c r="N23" s="16"/>
       <c r="O23" s="16"/>
     </row>
-    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="15" t="s">
         <v>65</v>
       </c>
@@ -1808,10 +1791,10 @@
         <v>0</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G24" s="17"/>
       <c r="L24" s="16"/>
@@ -1819,7 +1802,7 @@
       <c r="N24" s="16"/>
       <c r="O24" s="16"/>
     </row>
-    <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="15" t="s">
         <v>67</v>
       </c>
@@ -1833,10 +1816,10 @@
         <v>0</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G25" s="17"/>
       <c r="L25" s="16"/>
@@ -1844,7 +1827,7 @@
       <c r="N25" s="16"/>
       <c r="O25" s="16"/>
     </row>
-    <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="15" t="s">
         <v>68</v>
       </c>
@@ -1858,10 +1841,10 @@
         <v>0</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G26" s="17"/>
       <c r="L26" s="16"/>
@@ -1869,7 +1852,7 @@
       <c r="N26" s="16"/>
       <c r="O26" s="16"/>
     </row>
-    <row r="27" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="15" t="s">
         <v>69</v>
       </c>
@@ -1883,10 +1866,10 @@
         <v>0</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G27" s="17"/>
       <c r="L27" s="16"/>
@@ -1894,7 +1877,7 @@
       <c r="N27" s="16"/>
       <c r="O27" s="16"/>
     </row>
-    <row r="28" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="15" t="s">
         <v>70</v>
       </c>
@@ -1908,22 +1891,22 @@
         <v>0</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F28" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="G28" s="15" t="s">
         <v>121</v>
-      </c>
-      <c r="G28" s="15" t="s">
-        <v>122</v>
       </c>
       <c r="L28" s="16"/>
       <c r="M28" s="16"/>
       <c r="N28" s="16"/>
       <c r="O28" s="16"/>
     </row>
-    <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="15" t="s">
-        <v>72</v>
+        <v>131</v>
       </c>
       <c r="B29" s="15" t="s">
         <v>71</v>
@@ -1935,10 +1918,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J29" s="16">
         <v>1</v>
@@ -1951,9 +1934,9 @@
       <c r="N29" s="16"/>
       <c r="O29" s="16"/>
     </row>
-    <row r="30" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B30" s="15" t="s">
         <v>71</v>
@@ -1965,19 +1948,19 @@
         <v>0</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="L30" s="16"/>
       <c r="M30" s="16"/>
       <c r="N30" s="16"/>
       <c r="O30" s="16"/>
     </row>
-    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>71</v>
@@ -1989,19 +1972,19 @@
         <v>0</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="L31" s="16"/>
       <c r="M31" s="16"/>
       <c r="N31" s="16"/>
       <c r="O31" s="16"/>
     </row>
-    <row r="32" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>71</v>
@@ -2013,22 +1996,22 @@
         <v>0</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F32" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="G32" s="15" t="s">
         <v>126</v>
-      </c>
-      <c r="G32" s="15" t="s">
-        <v>127</v>
       </c>
       <c r="L32" s="16"/>
       <c r="M32" s="16"/>
       <c r="N32" s="16"/>
       <c r="O32" s="16"/>
     </row>
-    <row r="33" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>71</v>
@@ -2040,10 +2023,10 @@
         <v>0</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G33" s="17"/>
       <c r="L33" s="16"/>
@@ -2051,9 +2034,9 @@
       <c r="N33" s="16"/>
       <c r="O33" s="16"/>
     </row>
-    <row r="34" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>71</v>
@@ -2065,10 +2048,10 @@
         <v>0</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G34" s="17"/>
       <c r="L34" s="16"/>
@@ -2076,13 +2059,13 @@
       <c r="N34" s="16"/>
       <c r="O34" s="16"/>
     </row>
-    <row r="35" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="B35" s="15" t="s">
-        <v>79</v>
-      </c>
       <c r="C35" s="16">
         <v>1</v>
       </c>
@@ -2090,10 +2073,10 @@
         <v>0</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G35" s="17"/>
       <c r="L35" s="16"/>
@@ -2101,12 +2084,12 @@
       <c r="N35" s="16"/>
       <c r="O35" s="16"/>
     </row>
-    <row r="36" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="15" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C36" s="16">
         <v>1</v>
@@ -2115,10 +2098,10 @@
         <v>0</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G36" s="17"/>
       <c r="L36" s="16"/>
@@ -2126,7 +2109,7 @@
       <c r="N36" s="16"/>
       <c r="O36" s="16"/>
     </row>
-    <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E37" s="15"/>
       <c r="F37" s="17"/>
       <c r="G37" s="17"/>
@@ -2135,7 +2118,7 @@
       <c r="N37" s="16"/>
       <c r="O37" s="16"/>
     </row>
-    <row r="38" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="E38" s="15"/>
       <c r="F38" s="17"/>
       <c r="G38" s="17"/>
@@ -2144,294 +2127,294 @@
       <c r="N38" s="16"/>
       <c r="O38" s="16"/>
     </row>
-    <row r="39" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="18"/>
       <c r="M39" s="16"/>
     </row>
-    <row r="40" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="18"/>
       <c r="M40" s="16"/>
     </row>
-    <row r="41" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M41" s="16"/>
     </row>
-    <row r="42" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M42" s="16"/>
     </row>
-    <row r="43" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M43" s="16"/>
     </row>
-    <row r="44" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M44" s="16"/>
     </row>
-    <row r="45" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M45" s="16"/>
     </row>
-    <row r="46" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M46" s="16"/>
     </row>
-    <row r="47" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M47" s="16"/>
     </row>
-    <row r="48" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M48" s="16"/>
     </row>
-    <row r="49" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M49" s="16"/>
     </row>
-    <row r="50" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M50" s="16"/>
     </row>
-    <row r="51" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M51" s="16"/>
     </row>
-    <row r="52" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M52" s="16"/>
     </row>
-    <row r="53" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M53" s="16"/>
     </row>
-    <row r="54" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M54" s="16"/>
     </row>
-    <row r="55" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M55" s="16"/>
     </row>
-    <row r="56" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M56" s="16"/>
     </row>
-    <row r="57" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M57" s="16"/>
     </row>
-    <row r="58" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M58" s="16"/>
     </row>
-    <row r="59" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M59" s="16"/>
     </row>
-    <row r="60" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M60" s="16"/>
     </row>
-    <row r="61" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M61" s="16"/>
     </row>
-    <row r="62" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M62" s="16"/>
     </row>
-    <row r="63" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M63" s="16"/>
     </row>
-    <row r="64" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M64" s="16"/>
     </row>
-    <row r="65" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M65" s="16"/>
     </row>
-    <row r="66" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M66" s="16"/>
     </row>
-    <row r="67" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M67" s="16"/>
     </row>
-    <row r="68" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M68" s="16"/>
     </row>
-    <row r="69" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M69" s="16"/>
     </row>
-    <row r="70" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M70" s="16"/>
     </row>
-    <row r="71" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M71" s="16"/>
     </row>
-    <row r="72" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M72" s="16"/>
     </row>
-    <row r="73" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M73" s="16"/>
     </row>
-    <row r="74" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M74" s="16"/>
     </row>
-    <row r="75" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M75" s="16"/>
     </row>
-    <row r="76" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M76" s="16"/>
     </row>
-    <row r="77" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M77" s="16"/>
     </row>
-    <row r="78" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M78" s="16"/>
     </row>
-    <row r="79" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M79" s="16"/>
     </row>
-    <row r="80" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M80" s="16"/>
     </row>
-    <row r="81" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M81" s="16"/>
     </row>
-    <row r="82" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M82" s="16"/>
     </row>
-    <row r="83" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M83" s="16"/>
     </row>
-    <row r="84" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M84" s="16"/>
     </row>
-    <row r="85" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M85" s="16"/>
     </row>
-    <row r="86" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M86" s="16"/>
     </row>
-    <row r="87" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M87" s="16"/>
     </row>
-    <row r="88" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M88" s="16"/>
     </row>
-    <row r="89" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M89" s="16"/>
     </row>
-    <row r="90" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M90" s="16"/>
     </row>
-    <row r="91" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M91" s="16"/>
     </row>
-    <row r="92" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M92" s="16"/>
     </row>
-    <row r="93" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M93" s="16"/>
     </row>
-    <row r="94" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M94" s="16"/>
     </row>
-    <row r="95" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M95" s="16"/>
     </row>
-    <row r="96" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M96" s="16"/>
     </row>
-    <row r="97" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M97" s="16"/>
     </row>
-    <row r="98" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M98" s="16"/>
     </row>
-    <row r="99" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M99" s="16"/>
     </row>
-    <row r="100" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M100" s="16"/>
     </row>
-    <row r="101" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M101" s="16"/>
     </row>
-    <row r="102" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M102" s="16"/>
     </row>
-    <row r="103" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M103" s="16"/>
     </row>
-    <row r="104" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M104" s="16"/>
     </row>
-    <row r="105" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M105" s="16"/>
     </row>
-    <row r="106" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M106" s="16"/>
     </row>
-    <row r="107" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M107" s="16"/>
     </row>
-    <row r="108" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M108" s="16"/>
     </row>
-    <row r="109" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M109" s="16"/>
     </row>
-    <row r="110" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M110" s="16"/>
     </row>
-    <row r="111" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M111" s="16"/>
     </row>
-    <row r="112" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M112" s="16"/>
     </row>
-    <row r="113" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M113" s="16"/>
     </row>
-    <row r="114" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M114" s="16"/>
     </row>
-    <row r="115" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M115" s="16"/>
     </row>
-    <row r="116" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M116" s="16"/>
     </row>
-    <row r="117" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M117" s="16"/>
     </row>
-    <row r="118" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M118" s="16"/>
     </row>
-    <row r="119" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M119" s="16"/>
     </row>
-    <row r="120" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M120" s="16"/>
     </row>
-    <row r="121" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M121" s="16"/>
     </row>
-    <row r="122" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M122" s="16"/>
     </row>
-    <row r="123" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M123" s="16"/>
     </row>
-    <row r="124" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M124" s="16"/>
     </row>
-    <row r="125" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M125" s="16"/>
     </row>
-    <row r="126" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M126" s="16"/>
     </row>
-    <row r="127" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M127" s="16"/>
     </row>
-    <row r="128" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M128" s="16"/>
     </row>
-    <row r="129" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M129" s="16"/>
     </row>
-    <row r="130" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M130" s="16"/>
     </row>
-    <row r="131" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M131" s="16"/>
     </row>
-    <row r="132" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M132" s="16"/>
     </row>
-    <row r="133" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="13:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="M133" s="16"/>
     </row>
-    <row r="145" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="19"/>
       <c r="B145" s="19"/>
       <c r="C145" s="20"/>
@@ -2444,7 +2427,7 @@
       <c r="J145" s="16"/>
       <c r="K145" s="16"/>
     </row>
-    <row r="146" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="19"/>
       <c r="B146" s="19"/>
       <c r="C146" s="20"/>
@@ -2457,7 +2440,7 @@
       <c r="J146" s="16"/>
       <c r="K146" s="16"/>
     </row>
-    <row r="147" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="19"/>
       <c r="B147" s="19"/>
       <c r="C147" s="20"/>
@@ -2470,7 +2453,7 @@
       <c r="J147" s="16"/>
       <c r="K147" s="16"/>
     </row>
-    <row r="148" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="19"/>
       <c r="B148" s="19"/>
       <c r="C148" s="20"/>
@@ -2483,7 +2466,7 @@
       <c r="J148" s="16"/>
       <c r="K148" s="16"/>
     </row>
-    <row r="149" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="19"/>
       <c r="B149" s="19"/>
       <c r="C149" s="20"/>
@@ -2496,7 +2479,7 @@
       <c r="J149" s="20"/>
       <c r="K149" s="16"/>
     </row>
-    <row r="150" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="19"/>
       <c r="B150" s="19"/>
       <c r="C150" s="20"/>
@@ -2509,7 +2492,7 @@
       <c r="J150" s="20"/>
       <c r="K150" s="16"/>
     </row>
-    <row r="151" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="19"/>
       <c r="B151" s="19"/>
       <c r="C151" s="20"/>
@@ -2522,7 +2505,7 @@
       <c r="J151" s="20"/>
       <c r="K151" s="16"/>
     </row>
-    <row r="152" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="19"/>
       <c r="B152" s="19"/>
       <c r="C152" s="20"/>
@@ -2535,7 +2518,7 @@
       <c r="J152" s="20"/>
       <c r="K152" s="16"/>
     </row>
-    <row r="153" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="19"/>
       <c r="B153" s="19"/>
       <c r="C153" s="20"/>
@@ -2548,7 +2531,7 @@
       <c r="J153" s="16"/>
       <c r="K153" s="20"/>
     </row>
-    <row r="154" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="19"/>
       <c r="B154" s="19"/>
       <c r="C154" s="20"/>
@@ -2561,7 +2544,7 @@
       <c r="J154" s="16"/>
       <c r="K154" s="20"/>
     </row>
-    <row r="155" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="19"/>
       <c r="B155" s="19"/>
       <c r="C155" s="20"/>
@@ -2574,7 +2557,7 @@
       <c r="J155" s="16"/>
       <c r="K155" s="20"/>
     </row>
-    <row r="156" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="19"/>
       <c r="B156" s="19"/>
       <c r="C156" s="20"/>
@@ -2587,7 +2570,7 @@
       <c r="J156" s="16"/>
       <c r="K156" s="20"/>
     </row>
-    <row r="157" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:11" s="21" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="19"/>
       <c r="B157" s="19"/>
       <c r="C157" s="20"/>
@@ -2608,63 +2591,63 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{327D14A3-5FD1-442E-889F-ABD1F8B88941}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="34.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="24" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
         <v>55</v>
       </c>
       <c r="B2" s="15"/>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" s="15"/>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
         <v>60</v>
       </c>
       <c r="B4" s="15"/>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>66</v>
       </c>
       <c r="B5" s="15"/>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="15" t="s">
         <v>45</v>
       </c>
       <c r="B6" s="15"/>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
         <v>71</v>
       </c>
       <c r="B7" s="15"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="15" t="s">
         <v>39</v>
       </c>
       <c r="B8" s="15"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
         <v>51</v>
       </c>
@@ -2678,29 +2661,29 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDDDA012-88D7-4C64-AD5E-9CC7E5FD4B46}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="5" width="18.77734375" customWidth="1"/>
+    <col min="1" max="5" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="38.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
         <v>30</v>
       </c>
@@ -2717,7 +2700,7 @@
         <v>0.4375</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="24" t="s">
         <v>31</v>
       </c>
@@ -2734,7 +2717,7 @@
         <v>0.64583333333333337</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="24" t="s">
         <v>32</v>
       </c>
@@ -2751,7 +2734,7 @@
         <v>0.5625</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="24" t="s">
         <v>33</v>
       </c>
@@ -2776,32 +2759,32 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{726A2C25-0347-41F6-B5D5-DA1F7F6CAC15}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="27" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="27" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="27" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
         <v>37</v>
       </c>
@@ -2814,13 +2797,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95509931-205E-4233-97CE-08E7D34F8C4E}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="5" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="14"/>
       <c r="B1" s="24" t="s">
         <v>30</v>
@@ -2835,7 +2818,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="23" t="s">
         <v>55</v>
       </c>
@@ -2844,16 +2827,16 @@
       <c r="D2" s="16"/>
       <c r="E2" s="16"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
       <c r="E3" s="16"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="23" t="s">
         <v>60</v>
       </c>
@@ -2862,7 +2845,7 @@
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
         <v>66</v>
       </c>
@@ -2871,7 +2854,7 @@
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
         <v>45</v>
       </c>
@@ -2880,7 +2863,7 @@
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="23" t="s">
         <v>71</v>
       </c>
@@ -2889,7 +2872,7 @@
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="23" t="s">
         <v>39</v>
       </c>
@@ -2898,7 +2881,7 @@
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="23" t="s">
         <v>51</v>
       </c>
@@ -2915,12 +2898,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE249AB6-1E39-4F04-B76B-4EEF7346234E}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="23"/>
       <c r="B1" s="24" t="s">
         <v>34</v>
@@ -2935,7 +2918,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>55</v>
       </c>
@@ -2944,16 +2927,16 @@
       <c r="D2" s="16"/>
       <c r="E2" s="16"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="16"/>
       <c r="D3" s="16"/>
       <c r="E3" s="16"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
         <v>60</v>
       </c>
@@ -2962,7 +2945,7 @@
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
         <v>66</v>
       </c>
@@ -2971,7 +2954,7 @@
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>45</v>
       </c>
@@ -2980,7 +2963,7 @@
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>71</v>
       </c>
@@ -2989,7 +2972,7 @@
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
         <v>39</v>
       </c>
@@ -2998,7 +2981,7 @@
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
         <v>51</v>
       </c>
@@ -3015,18 +2998,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD6D2000-3325-493C-84D0-E8B832BF1752}">
   <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="29.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="14"/>
       <c r="B1" s="14" t="s">
         <v>55</v>
       </c>
       <c r="C1" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D1" s="14" t="s">
         <v>60</v>
@@ -3047,7 +3030,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>55</v>
       </c>
@@ -3060,9 +3043,9 @@
       <c r="H2" s="16"/>
       <c r="I2" s="16"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B3" s="28"/>
       <c r="C3" s="28"/>
@@ -3075,7 +3058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
         <v>60</v>
       </c>
@@ -3088,7 +3071,7 @@
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
         <v>66</v>
       </c>
@@ -3101,7 +3084,7 @@
       <c r="H5" s="16"/>
       <c r="I5" s="16"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>45</v>
       </c>
@@ -3114,7 +3097,7 @@
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>71</v>
       </c>
@@ -3127,7 +3110,7 @@
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
         <v>39</v>
       </c>
@@ -3140,7 +3123,7 @@
       <c r="H8" s="28"/>
       <c r="I8" s="16"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
         <v>51</v>
       </c>
@@ -3161,12 +3144,12 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20233A97-8339-4329-BFF1-D432565ECAD5}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="5" width="13.109375" customWidth="1"/>
+    <col min="2" max="5" width="13.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="23"/>
       <c r="B1" s="24" t="s">
         <v>34</v>
@@ -3181,7 +3164,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
         <v>30</v>
       </c>
@@ -3190,7 +3173,7 @@
       <c r="D2" s="16"/>
       <c r="E2" s="16"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="24" t="s">
         <v>31</v>
       </c>
@@ -3199,7 +3182,7 @@
       <c r="D3" s="16"/>
       <c r="E3" s="16"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="24" t="s">
         <v>32</v>
       </c>
@@ -3208,7 +3191,7 @@
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="24" t="s">
         <v>33</v>
       </c>

</xml_diff>